<commit_message>
Lawang/excel: quitar imagen del informe — solo texto y números (preferencia cliente)
- build_plan.py: eliminado el banner de portada y el import de imagen
- borrado assets/portada_sumba.png (huérfano)
- README actualizado

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/salida/Lamborghini_Sumba_Phase_I.xlsx
+++ b/excel/salida/Lamborghini_Sumba_Phase_I.xlsx
@@ -321,36 +321,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>4</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="6534150" cy="3657600"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -643,7 +613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:E81"/>
+  <dimension ref="B1:E68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -683,726 +653,714 @@
       <c r="D3" s="5" t="n"/>
       <c r="E3" s="5" t="n"/>
     </row>
-    <row r="4" ht="6" customHeight="1"/>
-    <row r="5" ht="24" customHeight="1"/>
-    <row r="6" ht="24" customHeight="1"/>
-    <row r="7" ht="24" customHeight="1"/>
-    <row r="8" ht="24" customHeight="1"/>
-    <row r="9" ht="24" customHeight="1"/>
-    <row r="10" ht="24" customHeight="1"/>
-    <row r="11" ht="24" customHeight="1"/>
-    <row r="12" ht="24" customHeight="1"/>
-    <row r="13" ht="24" customHeight="1"/>
-    <row r="14" ht="24" customHeight="1"/>
-    <row r="15" ht="24" customHeight="1"/>
-    <row r="16" ht="24" customHeight="1"/>
-    <row r="18" ht="8" customHeight="1"/>
-    <row r="19" ht="26" customHeight="1">
-      <c r="B19" s="6" t="inlineStr">
+    <row r="4" ht="10" customHeight="1"/>
+    <row r="5" ht="8" customHeight="1"/>
+    <row r="6" ht="26" customHeight="1">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>PROJECT SNAPSHOT — PHASE I</t>
         </is>
       </c>
-      <c r="C19" s="2" t="n"/>
-      <c r="D19" s="2" t="n"/>
-      <c r="E19" s="2" t="n"/>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Nº villas</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="n"/>
+      <c r="D7" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="E7" s="8" t="n"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Precio de venta por villa</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="n"/>
+      <c r="D8" s="12" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E8" s="11" t="n"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Superficie por villa</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="n"/>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>500 m²</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="n"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Ventas totales (GDV)</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="n"/>
+      <c r="D10" s="12" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="E10" s="11" t="n"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Inicio comercialización</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="n"/>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Mes 2 – 4</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="n"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Entrega estimada</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>Mes 12 – 14</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="n"/>
+    </row>
+    <row r="13" ht="8" customHeight="1"/>
+    <row r="14" ht="26" customHeight="1">
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>ESTADO DE RESULTADOS — PHASE I</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>CONCEPTO</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>CÁLCULO</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>IMPORTE</t>
+        </is>
+      </c>
+      <c r="E15" s="16" t="inlineStr">
+        <is>
+          <t>% S/ VENTAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Ventas de villas</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="inlineStr">
+        <is>
+          <t>10 × 1.000.000 €</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="E16" s="19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="B17" s="20" t="inlineStr">
+        <is>
+          <t>TOTAL INGRESOS</t>
+        </is>
+      </c>
+      <c r="C17" s="21" t="inlineStr"/>
+      <c r="D17" s="22" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="E17" s="23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Construcción</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="inlineStr"/>
+      <c r="D18" s="18" t="n">
+        <v>-3000000</v>
+      </c>
+      <c r="E18" s="19" t="n">
+        <v>-0.3</v>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>Suelo (adquisición)</t>
+        </is>
+      </c>
+      <c r="C19" s="24" t="inlineStr"/>
+      <c r="D19" s="12" t="n">
+        <v>-2000000</v>
+      </c>
+      <c r="E19" s="25" t="n">
+        <v>-0.2</v>
+      </c>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Nº villas</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="n"/>
-      <c r="D20" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="E20" s="8" t="n"/>
+          <t>Urbanización &amp; infraestructura</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="inlineStr"/>
+      <c r="D20" s="18" t="n">
+        <v>-500000</v>
+      </c>
+      <c r="E20" s="19" t="n">
+        <v>-0.05</v>
+      </c>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>Precio de venta por villa</t>
-        </is>
-      </c>
-      <c r="C21" s="11" t="n"/>
+          <t>Licencias &amp; permisos</t>
+        </is>
+      </c>
+      <c r="C21" s="24" t="inlineStr"/>
       <c r="D21" s="12" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="E21" s="11" t="n"/>
+        <v>-100000</v>
+      </c>
+      <c r="E21" s="25" t="n">
+        <v>-0.01</v>
+      </c>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Superficie por villa</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="n"/>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>500 m²</t>
-        </is>
-      </c>
-      <c r="E22" s="8" t="n"/>
+          <t>Nick Maltese Studio (diseño &amp; arq.)</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="inlineStr">
+        <is>
+          <t>8% s/ construcción</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="n">
+        <v>-240000</v>
+      </c>
+      <c r="E22" s="19" t="n">
+        <v>-0.024</v>
+      </c>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>Ventas totales (GDV)</t>
-        </is>
-      </c>
-      <c r="C23" s="11" t="n"/>
+          <t>Arquitecto local &amp; ingeniería</t>
+        </is>
+      </c>
+      <c r="C23" s="24" t="inlineStr"/>
       <c r="D23" s="12" t="n">
-        <v>10000000</v>
-      </c>
-      <c r="E23" s="11" t="n"/>
+        <v>-120000</v>
+      </c>
+      <c r="E23" s="25" t="n">
+        <v>-0.012</v>
+      </c>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Inicio comercialización</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="n"/>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>Mes 2 – 4</t>
-        </is>
-      </c>
-      <c r="E24" s="8" t="n"/>
+          <t>Otros profesionales técnicos</t>
+        </is>
+      </c>
+      <c r="C24" s="17" t="inlineStr"/>
+      <c r="D24" s="18" t="n">
+        <v>-80000</v>
+      </c>
+      <c r="E24" s="19" t="n">
+        <v>-0.008</v>
+      </c>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>Entrega estimada</t>
-        </is>
-      </c>
-      <c r="C25" s="11" t="n"/>
-      <c r="D25" s="13" t="inlineStr">
-        <is>
-          <t>Mes 12 – 14</t>
-        </is>
-      </c>
-      <c r="E25" s="11" t="n"/>
-    </row>
-    <row r="26" ht="8" customHeight="1"/>
-    <row r="27" ht="26" customHeight="1">
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>ESTADO DE RESULTADOS — PHASE I</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="n"/>
-      <c r="D27" s="2" t="n"/>
-      <c r="E27" s="2" t="n"/>
-    </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="B28" s="14" t="inlineStr">
-        <is>
-          <t>CONCEPTO</t>
-        </is>
-      </c>
-      <c r="C28" s="15" t="inlineStr">
-        <is>
-          <t>CÁLCULO</t>
-        </is>
-      </c>
-      <c r="D28" s="16" t="inlineStr">
-        <is>
-          <t>IMPORTE</t>
-        </is>
-      </c>
-      <c r="E28" s="16" t="inlineStr">
-        <is>
-          <t>% S/ VENTAS</t>
-        </is>
+          <t>Marketing &amp; branding</t>
+        </is>
+      </c>
+      <c r="C25" s="24" t="inlineStr"/>
+      <c r="D25" s="12" t="n">
+        <v>-150000</v>
+      </c>
+      <c r="E25" s="25" t="n">
+        <v>-0.015</v>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Comisiones comerciales</t>
+        </is>
+      </c>
+      <c r="C26" s="17" t="inlineStr">
+        <is>
+          <t>% de ventas</t>
+        </is>
+      </c>
+      <c r="D26" s="18" t="n">
+        <v>-300000</v>
+      </c>
+      <c r="E26" s="19" t="n">
+        <v>-0.03</v>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>Gastos legales &amp; notaría</t>
+        </is>
+      </c>
+      <c r="C27" s="24" t="inlineStr"/>
+      <c r="D27" s="12" t="n">
+        <v>-50000</v>
+      </c>
+      <c r="E27" s="25" t="n">
+        <v>-0.005</v>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Gastos administrativos</t>
+        </is>
+      </c>
+      <c r="C28" s="17" t="inlineStr"/>
+      <c r="D28" s="18" t="n">
+        <v>-50000</v>
+      </c>
+      <c r="E28" s="19" t="n">
+        <v>-0.005</v>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1">
-      <c r="B29" s="7" t="inlineStr">
-        <is>
-          <t>Ventas de villas</t>
-        </is>
-      </c>
-      <c r="C29" s="17" t="inlineStr">
-        <is>
-          <t>10 × 1.000.000 €</t>
-        </is>
-      </c>
-      <c r="D29" s="18" t="n">
-        <v>10000000</v>
-      </c>
-      <c r="E29" s="19" t="n">
-        <v>1</v>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>Seguros &amp; contingencias</t>
+        </is>
+      </c>
+      <c r="C29" s="24" t="inlineStr">
+        <is>
+          <t>% de ventas</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="n">
+        <v>-200000</v>
+      </c>
+      <c r="E29" s="25" t="n">
+        <v>-0.02</v>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="B30" s="20" t="inlineStr">
         <is>
-          <t>TOTAL INGRESOS</t>
+          <t>MARGEN OPERATIVO ANTES DE REPARTOS</t>
         </is>
       </c>
       <c r="C30" s="21" t="inlineStr"/>
       <c r="D30" s="22" t="n">
-        <v>10000000</v>
+        <v>3210000</v>
       </c>
       <c r="E30" s="23" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>Construcción</t>
-        </is>
-      </c>
-      <c r="C31" s="17" t="inlineStr"/>
-      <c r="D31" s="18" t="n">
-        <v>-3000000</v>
-      </c>
-      <c r="E31" s="19" t="n">
-        <v>-0.3</v>
-      </c>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="B32" s="10" t="inlineStr">
-        <is>
-          <t>Suelo (adquisición)</t>
-        </is>
-      </c>
-      <c r="C32" s="24" t="inlineStr"/>
-      <c r="D32" s="12" t="n">
-        <v>-2000000</v>
-      </c>
-      <c r="E32" s="25" t="n">
-        <v>-0.2</v>
-      </c>
+        <v>0.321</v>
+      </c>
+    </row>
+    <row r="31" ht="8" customHeight="1"/>
+    <row r="32" ht="26" customHeight="1">
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>REPARTO DEL BENEFICIO</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="n"/>
+      <c r="D32" s="2" t="n"/>
+      <c r="E32" s="2" t="n"/>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>Urbanización &amp; infraestructura</t>
-        </is>
-      </c>
-      <c r="C33" s="17" t="inlineStr"/>
+          <t>Tonino Lamborghini</t>
+        </is>
+      </c>
+      <c r="C33" s="17" t="inlineStr">
+        <is>
+          <t>3% del beneficio</t>
+        </is>
+      </c>
       <c r="D33" s="18" t="n">
-        <v>-500000</v>
-      </c>
-      <c r="E33" s="19" t="n">
-        <v>-0.05</v>
-      </c>
+        <v>-96300</v>
+      </c>
+      <c r="E33" s="8" t="n"/>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>Licencias &amp; permisos</t>
-        </is>
-      </c>
-      <c r="C34" s="24" t="inlineStr"/>
+          <t>Introducción de marca</t>
+        </is>
+      </c>
+      <c r="C34" s="24" t="inlineStr">
+        <is>
+          <t>1% del beneficio</t>
+        </is>
+      </c>
       <c r="D34" s="12" t="n">
-        <v>-100000</v>
-      </c>
-      <c r="E34" s="25" t="n">
-        <v>-0.01</v>
-      </c>
+        <v>-32100</v>
+      </c>
+      <c r="E34" s="11" t="n"/>
     </row>
     <row r="35" ht="20" customHeight="1">
-      <c r="B35" s="7" t="inlineStr">
-        <is>
-          <t>Nick Maltese Studio (diseño &amp; arq.)</t>
-        </is>
-      </c>
-      <c r="C35" s="17" t="inlineStr">
-        <is>
-          <t>8% s/ construcción</t>
-        </is>
-      </c>
-      <c r="D35" s="18" t="n">
-        <v>-240000</v>
-      </c>
-      <c r="E35" s="19" t="n">
-        <v>-0.024</v>
-      </c>
-    </row>
-    <row r="36" ht="20" customHeight="1">
-      <c r="B36" s="10" t="inlineStr">
-        <is>
-          <t>Arquitecto local &amp; ingeniería</t>
-        </is>
-      </c>
-      <c r="C36" s="24" t="inlineStr"/>
-      <c r="D36" s="12" t="n">
-        <v>-120000</v>
-      </c>
-      <c r="E36" s="25" t="n">
-        <v>-0.012</v>
-      </c>
-    </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="B37" s="7" t="inlineStr">
-        <is>
-          <t>Otros profesionales técnicos</t>
-        </is>
-      </c>
-      <c r="C37" s="17" t="inlineStr"/>
-      <c r="D37" s="18" t="n">
-        <v>-80000</v>
-      </c>
-      <c r="E37" s="19" t="n">
-        <v>-0.008</v>
-      </c>
-    </row>
-    <row r="38" ht="20" customHeight="1">
-      <c r="B38" s="10" t="inlineStr">
-        <is>
-          <t>Marketing &amp; branding</t>
-        </is>
-      </c>
-      <c r="C38" s="24" t="inlineStr"/>
-      <c r="D38" s="12" t="n">
-        <v>-150000</v>
-      </c>
-      <c r="E38" s="25" t="n">
-        <v>-0.015</v>
-      </c>
-    </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="B39" s="7" t="inlineStr">
-        <is>
-          <t>Comisiones comerciales</t>
-        </is>
-      </c>
-      <c r="C39" s="17" t="inlineStr">
-        <is>
-          <t>% de ventas</t>
-        </is>
-      </c>
-      <c r="D39" s="18" t="n">
-        <v>-300000</v>
-      </c>
-      <c r="E39" s="19" t="n">
-        <v>-0.03</v>
-      </c>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="B40" s="10" t="inlineStr">
-        <is>
-          <t>Gastos legales &amp; notaría</t>
-        </is>
-      </c>
-      <c r="C40" s="24" t="inlineStr"/>
-      <c r="D40" s="12" t="n">
-        <v>-50000</v>
-      </c>
-      <c r="E40" s="25" t="n">
-        <v>-0.005</v>
-      </c>
-    </row>
-    <row r="41" ht="20" customHeight="1">
-      <c r="B41" s="7" t="inlineStr">
-        <is>
-          <t>Gastos administrativos</t>
-        </is>
-      </c>
-      <c r="C41" s="17" t="inlineStr"/>
-      <c r="D41" s="18" t="n">
-        <v>-50000</v>
-      </c>
-      <c r="E41" s="19" t="n">
-        <v>-0.005</v>
-      </c>
-    </row>
-    <row r="42" ht="20" customHeight="1">
-      <c r="B42" s="10" t="inlineStr">
-        <is>
-          <t>Seguros &amp; contingencias</t>
-        </is>
-      </c>
-      <c r="C42" s="24" t="inlineStr">
-        <is>
-          <t>% de ventas</t>
-        </is>
-      </c>
-      <c r="D42" s="12" t="n">
-        <v>-200000</v>
-      </c>
-      <c r="E42" s="25" t="n">
-        <v>-0.02</v>
-      </c>
-    </row>
-    <row r="43" ht="20" customHeight="1">
-      <c r="B43" s="20" t="inlineStr">
-        <is>
-          <t>MARGEN OPERATIVO ANTES DE REPARTOS</t>
-        </is>
-      </c>
-      <c r="C43" s="21" t="inlineStr"/>
-      <c r="D43" s="22" t="n">
-        <v>3210000</v>
-      </c>
-      <c r="E43" s="23" t="n">
-        <v>0.321</v>
-      </c>
-    </row>
-    <row r="44" ht="8" customHeight="1"/>
-    <row r="45" ht="26" customHeight="1">
-      <c r="B45" s="6" t="inlineStr">
-        <is>
-          <t>REPARTO DEL BENEFICIO</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="n"/>
-      <c r="D45" s="2" t="n"/>
-      <c r="E45" s="2" t="n"/>
-    </row>
-    <row r="46" ht="20" customHeight="1">
-      <c r="B46" s="7" t="inlineStr">
-        <is>
-          <t>Tonino Lamborghini</t>
-        </is>
-      </c>
-      <c r="C46" s="17" t="inlineStr">
-        <is>
-          <t>3% del beneficio</t>
-        </is>
-      </c>
-      <c r="D46" s="18" t="n">
-        <v>-96300</v>
-      </c>
-      <c r="E46" s="8" t="n"/>
-    </row>
-    <row r="47" ht="20" customHeight="1">
-      <c r="B47" s="10" t="inlineStr">
-        <is>
-          <t>Introducción de marca</t>
-        </is>
-      </c>
-      <c r="C47" s="24" t="inlineStr">
-        <is>
-          <t>1% del beneficio</t>
-        </is>
-      </c>
-      <c r="D47" s="12" t="n">
-        <v>-32100</v>
-      </c>
-      <c r="E47" s="11" t="n"/>
-    </row>
-    <row r="48" ht="20" customHeight="1">
-      <c r="B48" s="20" t="inlineStr">
+      <c r="B35" s="20" t="inlineStr">
         <is>
           <t>BENEFICIO NETO PARA LAWANG (Fran &amp; Pablo)</t>
         </is>
       </c>
-      <c r="C48" s="26" t="n"/>
-      <c r="D48" s="22" t="n">
+      <c r="C35" s="26" t="n"/>
+      <c r="D35" s="22" t="n">
         <v>3081600</v>
       </c>
-      <c r="E48" s="26" t="n"/>
-    </row>
-    <row r="49" ht="8" customHeight="1"/>
-    <row r="50" ht="26" customHeight="1">
-      <c r="B50" s="6" t="inlineStr">
+      <c r="E35" s="26" t="n"/>
+    </row>
+    <row r="36" ht="8" customHeight="1"/>
+    <row r="37" ht="26" customHeight="1">
+      <c r="B37" s="6" t="inlineStr">
         <is>
           <t>MÉTRICAS CLAVE — PHASE I</t>
         </is>
       </c>
-      <c r="C50" s="2" t="n"/>
-      <c r="D50" s="2" t="n"/>
-      <c r="E50" s="2" t="n"/>
-    </row>
-    <row r="51" ht="18" customHeight="1">
-      <c r="B51" s="27" t="inlineStr">
+      <c r="C37" s="2" t="n"/>
+      <c r="D37" s="2" t="n"/>
+      <c r="E37" s="2" t="n"/>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="B38" s="27" t="inlineStr">
         <is>
           <t>VENTAS (GDV)</t>
         </is>
+      </c>
+      <c r="C38" s="5" t="n"/>
+      <c r="D38" s="5" t="n"/>
+      <c r="E38" s="5" t="n"/>
+    </row>
+    <row r="39" ht="36" customHeight="1">
+      <c r="B39" s="28" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="C39" s="5" t="n"/>
+      <c r="D39" s="5" t="n"/>
+      <c r="E39" s="5" t="n"/>
+    </row>
+    <row r="40" ht="6" customHeight="1"/>
+    <row r="41" ht="18" customHeight="1">
+      <c r="B41" s="27" t="inlineStr">
+        <is>
+          <t>BENEFICIO NETO LAWANG</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="n"/>
+      <c r="D41" s="5" t="n"/>
+      <c r="E41" s="5" t="n"/>
+    </row>
+    <row r="42" ht="36" customHeight="1">
+      <c r="B42" s="28" t="n">
+        <v>3081600</v>
+      </c>
+      <c r="C42" s="5" t="n"/>
+      <c r="D42" s="5" t="n"/>
+      <c r="E42" s="5" t="n"/>
+    </row>
+    <row r="43" ht="6" customHeight="1"/>
+    <row r="44" ht="18" customHeight="1">
+      <c r="B44" s="27" t="inlineStr">
+        <is>
+          <t>MARGEN NETO SOBRE VENTAS</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="n"/>
+      <c r="D44" s="5" t="n"/>
+      <c r="E44" s="5" t="n"/>
+    </row>
+    <row r="45" ht="36" customHeight="1">
+      <c r="B45" s="29" t="n">
+        <v>0.30816</v>
+      </c>
+      <c r="C45" s="5" t="n"/>
+      <c r="D45" s="5" t="n"/>
+      <c r="E45" s="5" t="n"/>
+    </row>
+    <row r="46" ht="6" customHeight="1"/>
+    <row r="47" ht="18" customHeight="1">
+      <c r="B47" s="27" t="inlineStr">
+        <is>
+          <t>ROI SOBRE COSTE TOTAL</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="n"/>
+      <c r="D47" s="5" t="n"/>
+      <c r="E47" s="5" t="n"/>
+    </row>
+    <row r="48" ht="36" customHeight="1">
+      <c r="B48" s="29" t="n">
+        <v>0.4538438880706922</v>
+      </c>
+      <c r="C48" s="5" t="n"/>
+      <c r="D48" s="5" t="n"/>
+      <c r="E48" s="5" t="n"/>
+    </row>
+    <row r="49" ht="6" customHeight="1"/>
+    <row r="50" ht="18" customHeight="1">
+      <c r="B50" s="27" t="inlineStr">
+        <is>
+          <t>ROI SOBRE INVERSIÓN TOTAL</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="n"/>
+      <c r="D50" s="5" t="n"/>
+      <c r="E50" s="5" t="n"/>
+    </row>
+    <row r="51" ht="36" customHeight="1">
+      <c r="B51" s="29" t="n">
+        <v>0.5135999999999999</v>
       </c>
       <c r="C51" s="5" t="n"/>
       <c r="D51" s="5" t="n"/>
       <c r="E51" s="5" t="n"/>
     </row>
-    <row r="52" ht="36" customHeight="1">
-      <c r="B52" s="28" t="n">
-        <v>10000000</v>
-      </c>
-      <c r="C52" s="5" t="n"/>
-      <c r="D52" s="5" t="n"/>
-      <c r="E52" s="5" t="n"/>
-    </row>
-    <row r="53" ht="6" customHeight="1"/>
-    <row r="54" ht="18" customHeight="1">
-      <c r="B54" s="27" t="inlineStr">
-        <is>
-          <t>BENEFICIO NETO LAWANG</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="n"/>
-      <c r="D54" s="5" t="n"/>
-      <c r="E54" s="5" t="n"/>
-    </row>
-    <row r="55" ht="36" customHeight="1">
-      <c r="B55" s="28" t="n">
-        <v>3081600</v>
-      </c>
-      <c r="C55" s="5" t="n"/>
-      <c r="D55" s="5" t="n"/>
-      <c r="E55" s="5" t="n"/>
-    </row>
-    <row r="56" ht="6" customHeight="1"/>
-    <row r="57" ht="18" customHeight="1">
-      <c r="B57" s="27" t="inlineStr">
-        <is>
-          <t>MARGEN NETO SOBRE VENTAS</t>
-        </is>
-      </c>
-      <c r="C57" s="5" t="n"/>
-      <c r="D57" s="5" t="n"/>
-      <c r="E57" s="5" t="n"/>
-    </row>
-    <row r="58" ht="36" customHeight="1">
-      <c r="B58" s="29" t="n">
-        <v>0.30816</v>
-      </c>
-      <c r="C58" s="5" t="n"/>
-      <c r="D58" s="5" t="n"/>
-      <c r="E58" s="5" t="n"/>
-    </row>
-    <row r="59" ht="6" customHeight="1"/>
-    <row r="60" ht="18" customHeight="1">
-      <c r="B60" s="27" t="inlineStr">
-        <is>
-          <t>ROI SOBRE COSTE TOTAL</t>
-        </is>
-      </c>
-      <c r="C60" s="5" t="n"/>
-      <c r="D60" s="5" t="n"/>
-      <c r="E60" s="5" t="n"/>
-    </row>
-    <row r="61" ht="36" customHeight="1">
-      <c r="B61" s="29" t="n">
-        <v>0.4538438880706922</v>
-      </c>
-      <c r="C61" s="5" t="n"/>
-      <c r="D61" s="5" t="n"/>
-      <c r="E61" s="5" t="n"/>
-    </row>
-    <row r="62" ht="6" customHeight="1"/>
-    <row r="63" ht="18" customHeight="1">
-      <c r="B63" s="27" t="inlineStr">
-        <is>
-          <t>ROI SOBRE INVERSIÓN TOTAL</t>
-        </is>
-      </c>
-      <c r="C63" s="5" t="n"/>
-      <c r="D63" s="5" t="n"/>
-      <c r="E63" s="5" t="n"/>
-    </row>
-    <row r="64" ht="36" customHeight="1">
-      <c r="B64" s="29" t="n">
-        <v>0.5135999999999999</v>
-      </c>
-      <c r="C64" s="5" t="n"/>
-      <c r="D64" s="5" t="n"/>
-      <c r="E64" s="5" t="n"/>
-    </row>
-    <row r="65" ht="6" customHeight="1"/>
-    <row r="66" ht="8" customHeight="1"/>
-    <row r="67" ht="26" customHeight="1">
-      <c r="B67" s="6" t="inlineStr">
+    <row r="52" ht="6" customHeight="1"/>
+    <row r="53" ht="8" customHeight="1"/>
+    <row r="54" ht="26" customHeight="1">
+      <c r="B54" s="6" t="inlineStr">
         <is>
           <t>CASH FLOW ESTIMADO — PHASE I</t>
         </is>
       </c>
-      <c r="C67" s="2" t="n"/>
-      <c r="D67" s="2" t="n"/>
-      <c r="E67" s="2" t="n"/>
-    </row>
-    <row r="68" ht="18" customHeight="1">
-      <c r="B68" s="14" t="inlineStr">
+      <c r="C54" s="2" t="n"/>
+      <c r="D54" s="2" t="n"/>
+      <c r="E54" s="2" t="n"/>
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="B55" s="14" t="inlineStr">
         <is>
           <t>HITO</t>
         </is>
       </c>
-      <c r="C68" s="15" t="inlineStr">
+      <c r="C55" s="15" t="inlineStr">
         <is>
           <t>MES</t>
         </is>
       </c>
-      <c r="D68" s="16" t="inlineStr">
+      <c r="D55" s="16" t="inlineStr">
         <is>
           <t>FLUJO</t>
         </is>
       </c>
-      <c r="E68" s="16" t="inlineStr">
+      <c r="E55" s="16" t="inlineStr">
         <is>
           <t>ACUMULADO</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="20" customHeight="1">
-      <c r="B69" s="7" t="inlineStr">
+    <row r="56" ht="20" customHeight="1">
+      <c r="B56" s="7" t="inlineStr">
         <is>
           <t>Preventas &amp; Reservas (30%)</t>
         </is>
       </c>
-      <c r="C69" s="30" t="inlineStr">
+      <c r="C56" s="30" t="inlineStr">
         <is>
           <t>2 – 4</t>
         </is>
       </c>
-      <c r="D69" s="18" t="n">
+      <c r="D56" s="18" t="n">
         <v>3000000</v>
       </c>
-      <c r="E69" s="31" t="n">
+      <c r="E56" s="31" t="n">
         <v>3000000</v>
       </c>
     </row>
-    <row r="70" ht="20" customHeight="1">
-      <c r="B70" s="10" t="inlineStr">
+    <row r="57" ht="20" customHeight="1">
+      <c r="B57" s="10" t="inlineStr">
         <is>
           <t>Inicio construcción</t>
         </is>
       </c>
-      <c r="C70" s="32" t="inlineStr">
+      <c r="C57" s="32" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="D70" s="12" t="n">
+      <c r="D57" s="12" t="n">
         <v>-1500000</v>
       </c>
-      <c r="E70" s="33" t="n">
+      <c r="E57" s="33" t="n">
         <v>1500000</v>
       </c>
     </row>
-    <row r="71" ht="20" customHeight="1">
-      <c r="B71" s="7" t="inlineStr">
+    <row r="58" ht="20" customHeight="1">
+      <c r="B58" s="7" t="inlineStr">
         <is>
           <t>Avance obra 30%</t>
         </is>
       </c>
-      <c r="C71" s="30" t="inlineStr">
+      <c r="C58" s="30" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="D71" s="18" t="n">
+      <c r="D58" s="18" t="n">
         <v>-1200000</v>
       </c>
-      <c r="E71" s="31" t="n">
+      <c r="E58" s="31" t="n">
         <v>300000</v>
       </c>
     </row>
-    <row r="72" ht="20" customHeight="1">
-      <c r="B72" s="10" t="inlineStr">
+    <row r="59" ht="20" customHeight="1">
+      <c r="B59" s="10" t="inlineStr">
         <is>
           <t>Avance obra 60%</t>
         </is>
       </c>
-      <c r="C72" s="32" t="inlineStr">
+      <c r="C59" s="32" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="D72" s="12" t="n">
+      <c r="D59" s="12" t="n">
         <v>-1000000</v>
       </c>
-      <c r="E72" s="33" t="n">
+      <c r="E59" s="33" t="n">
         <v>-700000</v>
       </c>
     </row>
-    <row r="73" ht="20" customHeight="1">
-      <c r="B73" s="7" t="inlineStr">
+    <row r="60" ht="20" customHeight="1">
+      <c r="B60" s="7" t="inlineStr">
         <is>
           <t>Avance obra 90%</t>
         </is>
       </c>
-      <c r="C73" s="30" t="inlineStr">
+      <c r="C60" s="30" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="D73" s="18" t="n">
+      <c r="D60" s="18" t="n">
         <v>-800000</v>
       </c>
-      <c r="E73" s="31" t="n">
+      <c r="E60" s="31" t="n">
         <v>-1500000</v>
       </c>
     </row>
-    <row r="74" ht="20" customHeight="1">
-      <c r="B74" s="10" t="inlineStr">
+    <row r="61" ht="20" customHeight="1">
+      <c r="B61" s="10" t="inlineStr">
         <is>
           <t>Entrega &amp; escrituración (70%)</t>
         </is>
       </c>
-      <c r="C74" s="32" t="inlineStr">
+      <c r="C61" s="32" t="inlineStr">
         <is>
           <t>12 – 14</t>
         </is>
       </c>
-      <c r="D74" s="12" t="n">
+      <c r="D61" s="12" t="n">
         <v>6581600</v>
       </c>
-      <c r="E74" s="33" t="n">
+      <c r="E61" s="33" t="n">
         <v>5081600</v>
       </c>
     </row>
-    <row r="75" ht="8" customHeight="1"/>
-    <row r="76" ht="26" customHeight="1">
-      <c r="B76" s="6" t="inlineStr">
+    <row r="62" ht="8" customHeight="1"/>
+    <row r="63" ht="26" customHeight="1">
+      <c r="B63" s="6" t="inlineStr">
         <is>
           <t>VALOR DEL SUELO</t>
         </is>
       </c>
-      <c r="C76" s="2" t="n"/>
-      <c r="D76" s="2" t="n"/>
-      <c r="E76" s="2" t="n"/>
-    </row>
-    <row r="77" ht="20" customHeight="1">
-      <c r="B77" s="7" t="inlineStr">
+      <c r="C63" s="2" t="n"/>
+      <c r="D63" s="2" t="n"/>
+      <c r="E63" s="2" t="n"/>
+    </row>
+    <row r="64" ht="20" customHeight="1">
+      <c r="B64" s="7" t="inlineStr">
         <is>
           <t>Coste de adquisición</t>
         </is>
       </c>
-      <c r="C77" s="17" t="inlineStr">
+      <c r="C64" s="17" t="inlineStr">
         <is>
           <t>20000 m² · 100 €/m²</t>
         </is>
       </c>
-      <c r="D77" s="18" t="n">
+      <c r="D64" s="18" t="n">
         <v>2000000</v>
       </c>
-      <c r="E77" s="8" t="n"/>
-    </row>
-    <row r="78" ht="20" customHeight="1">
-      <c r="B78" s="10" t="inlineStr">
+      <c r="E64" s="8" t="n"/>
+    </row>
+    <row r="65" ht="20" customHeight="1">
+      <c r="B65" s="10" t="inlineStr">
         <is>
           <t>Valor potencial del suelo</t>
         </is>
       </c>
-      <c r="C78" s="24" t="inlineStr">
+      <c r="C65" s="24" t="inlineStr">
         <is>
           <t>20000 m² × 200 €/m²</t>
         </is>
       </c>
-      <c r="D78" s="12" t="n">
+      <c r="D65" s="12" t="n">
         <v>4000000</v>
       </c>
-      <c r="E78" s="11" t="n"/>
-    </row>
-    <row r="79" ht="20" customHeight="1">
-      <c r="B79" s="20" t="inlineStr">
+      <c r="E65" s="11" t="n"/>
+    </row>
+    <row r="66" ht="20" customHeight="1">
+      <c r="B66" s="20" t="inlineStr">
         <is>
           <t>Plusvalía estimada</t>
         </is>
       </c>
-      <c r="C79" s="26" t="n"/>
-      <c r="D79" s="22" t="n">
+      <c r="C66" s="26" t="n"/>
+      <c r="D66" s="22" t="n">
         <v>2000000</v>
       </c>
-      <c r="E79" s="26" t="n"/>
-    </row>
-    <row r="81">
-      <c r="B81" s="34" t="inlineStr">
+      <c r="E66" s="26" t="n"/>
+    </row>
+    <row r="68">
+      <c r="B68" s="34" t="inlineStr">
         <is>
           <t>AxisWorks · Documento de inversión confidencial — Lawang Estate</t>
         </is>
@@ -1410,28 +1368,27 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="B64:E64"/>
-    <mergeCell ref="B55:E55"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="B68:E68"/>
     <mergeCell ref="B51:E51"/>
-    <mergeCell ref="B76:E76"/>
+    <mergeCell ref="B32:E32"/>
     <mergeCell ref="B45:E45"/>
     <mergeCell ref="B63:E63"/>
+    <mergeCell ref="B41:E41"/>
     <mergeCell ref="B50:E50"/>
     <mergeCell ref="B54:E54"/>
     <mergeCell ref="B3:E3"/>
-    <mergeCell ref="B81:E81"/>
-    <mergeCell ref="B27:E27"/>
-    <mergeCell ref="B58:E58"/>
-    <mergeCell ref="B52:E52"/>
+    <mergeCell ref="B47:E47"/>
+    <mergeCell ref="B48:E48"/>
+    <mergeCell ref="B39:E39"/>
     <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B60:E60"/>
-    <mergeCell ref="B67:E67"/>
-    <mergeCell ref="B61:E61"/>
+    <mergeCell ref="B42:E42"/>
+    <mergeCell ref="B14:E14"/>
     <mergeCell ref="B1:E1"/>
-    <mergeCell ref="B57:E57"/>
-    <mergeCell ref="B19:E19"/>
+    <mergeCell ref="B38:E38"/>
+    <mergeCell ref="B44:E44"/>
+    <mergeCell ref="B37:E37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>